<commit_message>
Lower CTTX Managed Service Retainer to R1,500/month per Gerhard's instruction
Was R4,500/month (mid-point of the R3,500-5,500 range). Recommended monthly recurring drops from R13,343 to R9,893, monthly saving vs Herotel rises from R4,762.60 to R8,212.60.

Payback tightens from 1 year 7 months to 1 year 0 months. Total 5-year saving rises from R316,855 to R559,732 - a materially stronger case for the R334K build investment, which was the stated goal.
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_5Year_Business_Case.xlsx
+++ b/proposals/Barefoot_5Year_Business_Case.xlsx
@@ -1863,14 +1863,14 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Managed Service Retainer (mid-tier of R3,500-R5,500 range)</t>
+          <t>Managed Service Retainer (remote monitoring, maintenance, support)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>5175</v>
+        <v>1725</v>
       </c>
       <c r="D23" s="6" t="n"/>
     </row>
@@ -2498,12 +2498,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>R4,500/month excl. VAT</t>
+          <t>R1,500/month excl. VAT</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t>Mid-point of CTTX's R3,500-R5,500/month range for a system this complex (mast, solar/battery, 30 radios).</t>
+          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the R334K build investment.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lower Vodacom Business Connect markup to 20% (was 25%) per Gerhard's instruction
Client price for the 100Mbps MRC drops from R8,168.00 to R7,841.16/month incl VAT (cost basis stays confidential, unchanged from the Notion pricing master). Combined with the R1,500 retainer, recommended monthly recurring is now R9,566.16 (was R9,893.00).

Payback stays at 1 year flat (unchanged - the tighter monthly saving of R8,539.44 vs R8,212.60 actually improves it marginally but not enough to shift the year-boundary). Total 5-year saving rises slightly to R582,741 (was R559,732).

Note: this lowers CTTX's own margin on the recurring line from R1,421/month to R1,136.40/month (ex VAT, internal - never shown in the client-facing file). The larger open question - zero markup currently on the R225,834 hardware+infrastructure portion of the CAPEX build - is still unresolved and flagged separately.
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_5Year_Business_Case.xlsx
+++ b/proposals/Barefoot_5Year_Business_Case.xlsx
@@ -1792,10 +1792,10 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>7103</v>
+        <v>6818.4</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>8168</v>
+        <v>7841.16</v>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add ROI row measured against Herotel spend avoided
New row on tab 4: ROI % = cumulative savings / total upfront cash outlay (R358,599 = R355K build + R3,599 Vodacom NRC), shown year by year alongside the existing Rand savings row. 5-Year ROI headline added to tab 1.

Year-by-year: -39.4% (Y0) -> -6.0% (Y1) -> 30.1% (Y2) -> 69.1% (Y3) -> 111.2% (Y4) -> 156.7% (Y5). Crosses into positive return partway through Year 2, consistent with the 1yr-2mo payback point already on the sheet.
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_5Year_Business_Case.xlsx
+++ b/proposals/Barefoot_5Year_Business_Case.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="&quot;R&quot;#,##0.00;(&quot;R&quot;#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +108,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
@@ -182,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -217,21 +223,26 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -778,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -797,7 +808,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
         <is>
           <t>Why build a private carrier-grade network instead of continuing to rent one, month after month, forever.</t>
         </is>
@@ -832,7 +843,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Right now the lodge pays a monthly bill to Herotel forever, for equipment it will never own, on a network it does not control. This proposal is the alternative: pay once to build a private network on your own engineered mast, then pay a much smaller monthly fee for the carrier link that feeds it. The network is built to run for 10 years, and CTTX supports it for that whole period.</t>
         </is>
@@ -853,7 +864,7 @@
           <t>One-time build cost (infrastructure, owned by the lodge)</t>
         </is>
       </c>
-      <c r="E14" s="31">
+      <c r="E14" s="33">
         <f>'2. Network Build Investment'!C6</f>
         <v/>
       </c>
@@ -864,7 +875,7 @@
           <t>Current Herotel monthly bill (connectivity + rented Wi-Fi equipment)</t>
         </is>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="33">
         <f>'3. Monthly Cost Comparison'!C11</f>
         <v/>
       </c>
@@ -875,7 +886,7 @@
           <t>New monthly bill once built (Vodacom link + CTTX monitoring - recommended)</t>
         </is>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="33">
         <f>'3. Monthly Cost Comparison'!C26</f>
         <v/>
       </c>
@@ -886,7 +897,7 @@
           <t>Monthly saving once built</t>
         </is>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="33">
         <f>E15-E16</f>
         <v/>
       </c>
@@ -897,8 +908,8 @@
           <t>Time to pay back the build cost</t>
         </is>
       </c>
-      <c r="E18" s="32">
-        <f>'4. 5-Year Cash Flow'!B28</f>
+      <c r="E18" s="34">
+        <f>'4. 5-Year Cash Flow'!B29</f>
         <v/>
       </c>
     </row>
@@ -908,80 +919,92 @@
           <t>Total saved over 5 years vs staying with Herotel</t>
         </is>
       </c>
-      <c r="E19" s="31">
-        <f>'4. 5-Year Cash Flow'!I30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="E19" s="33">
+        <f>'4. 5-Year Cash Flow'!I31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>5-Year Return on Investment</t>
+        </is>
+      </c>
+      <c r="E20" s="35">
+        <f>'4. 5-Year Cash Flow'!I32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Why This Makes Sense Over 10 Years</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>1. The lodge currently pays for connectivity AND for the right to use someone else's Wi-Fi equipment, every month, indefinitely. Nothing is ever owned.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>2. The existing backhaul radios are mounted on a leaning gum pole - not an engineered structure. That is a physical failure risk, separate from the cost problem.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>3. Building a private network converts a forever-rising monthly rental into a one-time build cost plus a much smaller ongoing carrier fee for just the connectivity - the Wi-Fi equipment, the mast, and the solar power all become the lodge's own asset.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="29" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>4. CTTX designs, builds, and supports this network for an expected 10-year working life - see tab 5 for what that support includes and excludes.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>5. See tab 4 for the year-by-year numbers: the build cost is recovered from the monthly saving within the payback period shown above, and every month after that is money the lodge keeps instead of sending to a telecoms reseller.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
         <is>
           <t>Full cost detail: tab 2 (build cost), tab 3 (monthly comparison), tab 4 (5-year cash flow), tab 5 (assumptions - read this before trusting any number on this page).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A24:F24"/>
+  <mergeCells count="19">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A9:F11"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A9:F11"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1981,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2337,99 +2360,141 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Return on Investment (cumulative savings vs. Herotel, as % of total upfront cash outlay)</t>
+        </is>
+      </c>
+      <c r="B21" s="24">
+        <f>B20/$B$17</f>
+        <v/>
+      </c>
+      <c r="C21" s="24">
+        <f>C20/$B$17</f>
+        <v/>
+      </c>
+      <c r="D21" s="24">
+        <f>D20/$B$17</f>
+        <v/>
+      </c>
+      <c r="E21" s="24">
+        <f>E20/$B$17</f>
+        <v/>
+      </c>
+      <c r="F21" s="24">
+        <f>F20/$B$17</f>
+        <v/>
+      </c>
+      <c r="G21" s="24">
+        <f>G20/$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Payback Calculation</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Last year cumulative savings still negative or zero (position in range)</t>
-        </is>
-      </c>
-      <c r="B23" s="24">
-        <f>MATCH(0,B20:G20,1)</f>
-        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>That year number</t>
-        </is>
-      </c>
-      <c r="B24" s="24">
-        <f>INDEX(B6:G6,B23)</f>
+          <t>Last year cumulative savings still negative or zero (position in range)</t>
+        </is>
+      </c>
+      <c r="B24" s="25">
+        <f>MATCH(0,B20:G20,1)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Cumulative savings at that year</t>
-        </is>
-      </c>
-      <c r="B25" s="22">
-        <f>INDEX(B20:G20,B23)</f>
+          <t>That year number</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>INDEX(B6:G6,B24)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Cumulative savings the following year</t>
+          <t>Cumulative savings at that year</t>
         </is>
       </c>
       <c r="B26" s="22">
-        <f>INDEX(B20:G20,B23+1)</f>
+        <f>INDEX(B20:G20,B24)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>Cumulative savings the following year</t>
+        </is>
+      </c>
+      <c r="B27" s="22">
+        <f>INDEX(B20:G20,B24+1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>Payback point (years, decimal)</t>
         </is>
       </c>
-      <c r="B27" s="25">
-        <f>B24+(-B25)/(B26-B25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="B28" s="26">
+        <f>B25+(-B26)/(B27-B26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Payback point (plain English)</t>
         </is>
       </c>
-      <c r="B28" s="26">
-        <f>TEXT(INT(B27),"0")&amp;" years, "&amp;TEXT(ROUND((B27-INT(B27))*12,0),"0")&amp;" months"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="B29" s="27">
+        <f>TEXT(INT(B28),"0")&amp;" years, "&amp;TEXT(ROUND((B28-INT(B28))*12,0),"0")&amp;" months"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Total 5-year saving vs Herotel (recommended path)</t>
         </is>
       </c>
-      <c r="I30" s="27">
+      <c r="I31" s="28">
         <f>G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>5-Year ROI (total saving as % of total upfront cash outlay)</t>
+        </is>
+      </c>
+      <c r="I32" s="29">
+        <f>G21</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="C4:H4"/>
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2465,12 +2530,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -2492,7 +2557,7 @@
           <t>8% p.a.</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>Not confirmed by either party - a typical CPI-linked telecom escalation in South Africa. Editable on tab 4; change it and every formula recalculates.</t>
         </is>
@@ -2509,7 +2574,7 @@
           <t>15%</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>Current South African VAT rate.</t>
         </is>
@@ -2526,7 +2591,7 @@
           <t>R1,500/month excl. VAT</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
         </is>
@@ -2543,7 +2608,7 @@
           <t>24 months</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Standard Vodacom Business Connect contract term. The network's physical life (10 years) is longer than this contract term - Vodacom connectivity is expected to be renewed at then-current rates.</t>
         </is>
@@ -2557,35 +2622,35 @@
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
         </is>
@@ -2599,21 +2664,21 @@
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>Years 1-3: monthly remote monitoring, quarterly on-site maintenance, 24/7 emergency support, proactive performance reporting, warranty-covered equipment troubleshooting/replacement.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Years 4-10: ongoing remote monitoring, annual on-site maintenance/assessment, 24/7 support continuation, planned technology refresh, performance reporting.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
         </is>
@@ -2627,35 +2692,35 @@
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
         </is>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="29" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="29" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>Any scope beyond the confirmed coverage zones (28 subscriber sites) without a signed change order.</t>
         </is>

</xml_diff>

<commit_message>
Correct Barefoot financial case: same clock, upfront included, locked pricing
The cash-flow model charged the current provider a full year of bills in
year 0 while giving the CTTX path none, and escalated CTTX's monthly fee
despite the proposal stating it is locked for the 36-month term. Both
paths now start at month 0 with the R358,599 upfront as the CTTX line's
origin; CTTX monthly is flat for 36 months, then 8%.

Payback 2 yr 10 mo (was 1 yr 1 mo); 5-year ROI 98% (was 169%); adds the
36-month-term comparison and the zero-escalation sensitivity. Workbook,
HTML, PDF and chart updated; rule recorded as decision 16.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_5Year_Business_Case.xlsx
+++ b/proposals/Barefoot_5Year_Business_Case.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="1. Business Case" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. Network Build Investment" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Monthly Cost Comparison" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. 5-Year Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5. Assumptions &amp; Scope" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2. Network Build Investment" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3. Monthly Cost Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4. 5-Year Cash Flow" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5. Assumptions &amp; Scope" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -188,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -227,6 +228,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="16" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -323,6 +325,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
   <chart>
     <title>
       <tx>
@@ -808,7 +811,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="32" t="inlineStr">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>Why build a private carrier-grade network instead of continuing to rent one, month after month, forever.</t>
         </is>
@@ -843,7 +846,7 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Right now the lodge pays a monthly bill to Herotel forever, for equipment it will never own, on a network it does not control. This proposal is the alternative: pay once to build a private network on your own engineered mast, then pay a much smaller monthly fee for the carrier link that feeds it. The network is built to run for 10 years, and CTTX supports it for that whole period.</t>
         </is>
@@ -864,7 +867,7 @@
           <t>One-time build cost (infrastructure, owned by the lodge)</t>
         </is>
       </c>
-      <c r="E14" s="33">
+      <c r="E14" s="34">
         <f>'2. Network Build Investment'!C6</f>
         <v/>
       </c>
@@ -875,7 +878,7 @@
           <t>Current Herotel monthly bill (connectivity + rented Wi-Fi equipment)</t>
         </is>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="34">
         <f>'3. Monthly Cost Comparison'!C11</f>
         <v/>
       </c>
@@ -886,7 +889,7 @@
           <t>New monthly bill once built (Vodacom link + CTTX monitoring - recommended)</t>
         </is>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="34">
         <f>'3. Monthly Cost Comparison'!C26</f>
         <v/>
       </c>
@@ -897,7 +900,7 @@
           <t>Monthly saving once built</t>
         </is>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="34">
         <f>E15-E16</f>
         <v/>
       </c>
@@ -908,7 +911,7 @@
           <t>Time to pay back the build cost</t>
         </is>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="35">
         <f>'4. 5-Year Cash Flow'!B29</f>
         <v/>
       </c>
@@ -919,8 +922,8 @@
           <t>Total saved over 5 years vs staying with Herotel</t>
         </is>
       </c>
-      <c r="E19" s="33">
-        <f>'4. 5-Year Cash Flow'!I31</f>
+      <c r="E19" s="34">
+        <f>'4. 5-Year Cash Flow'!I36</f>
         <v/>
       </c>
     </row>
@@ -930,8 +933,8 @@
           <t>5-Year Return on Investment</t>
         </is>
       </c>
-      <c r="E20" s="35">
-        <f>'4. 5-Year Cash Flow'!I32</f>
+      <c r="E20" s="36">
+        <f>'4. 5-Year Cash Flow'!I37</f>
         <v/>
       </c>
     </row>
@@ -943,35 +946,35 @@
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>1. The lodge currently pays for connectivity AND for the right to use someone else's Wi-Fi equipment, every month, indefinitely. Nothing is ever owned.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>2. The existing backhaul radios are mounted on a leaning gum pole - not an engineered structure. That is a physical failure risk, separate from the cost problem.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>3. Building a private network converts a forever-rising monthly rental into a one-time build cost plus a much smaller ongoing carrier fee for just the connectivity - the Wi-Fi equipment, the mast, and the solar power all become the lodge's own asset.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>4. CTTX designs, builds, and supports this network for an expected 10-year working life - see tab 5 for what that support includes and excludes.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>5. See tab 4 for the year-by-year numbers: the build cost is recovered from the monthly saving within the payback period shown above, and every month after that is money the lodge keeps instead of sending to a telecoms reseller.</t>
         </is>
@@ -1016,8 +1019,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D62"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1677,14 +1693,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
@@ -1998,14 +2014,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -2024,17 +2040,17 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="64" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Year 0 = build year (deposit and construction). Years 1-5 are projected here deliberately, rather than compounding the escalation assumption out to a full decade. The network's engineered/expected working life is longer (see tab 5) and CTTX's support commitment runs 10 years - this cash flow is the near-term financial case, not a claim about how long the equipment lasts. All figures incl. VAT.</t>
+          <t>Year 0 = the day the build is paid for. Both paths start paying their monthly bills from month 1, so the two lines are compared on the same clock: the current provider is NOT charged a year of bills before the build, and CTTX is NOT given a free year. Years 1-5 are projected here deliberately, rather than compounding the escalation assumption out to a full decade. The network's engineered/expected working life is longer (see tab 5) and CTTX's support commitment runs 10 years - this cash flow is the near-term financial case, not a claim about how long the equipment lasts. All figures incl. VAT.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>Annual escalation rate (applied to both Herotel and Vodacom monthly fees)</t>
+          <t>Annual escalation rate (current provider from year 2; CTTX only after the 36-month locked term, i.e. from year 4)</t>
         </is>
       </c>
       <c r="B4" s="20" t="n">
@@ -2081,15 +2097,14 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Herotel monthly bill (escalated)</t>
-        </is>
-      </c>
-      <c r="B8" s="22">
+          <t>Herotel monthly bill (year 1 = today's bill; escalated from year 2)</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="22">
         <f>'3. Monthly Cost Comparison'!$C$11</f>
-        <v/>
-      </c>
-      <c r="C8" s="22">
-        <f>B8*(1+$B$4)</f>
         <v/>
       </c>
       <c r="D8" s="22">
@@ -2233,7 +2248,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>CTTX monthly recurring (Vodacom + Retainer, escalated)</t>
+          <t>CTTX monthly recurring (Vodacom + Retainer; locked for the 36-month term, escalated from year 4)</t>
         </is>
       </c>
       <c r="B15" s="22" t="n">
@@ -2244,11 +2259,11 @@
         <v/>
       </c>
       <c r="D15" s="22">
-        <f>C15*(1+$B$4)</f>
+        <f>C15</f>
         <v/>
       </c>
       <c r="E15" s="22">
-        <f>D15*(1+$B$4)</f>
+        <f>D15</f>
         <v/>
       </c>
       <c r="F15" s="22">
@@ -2465,29 +2480,70 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Over the 36-month agreement term (end of year 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Paid to Herotel over 36 months (if nothing changes)</t>
+        </is>
+      </c>
+      <c r="B32" s="22">
+        <f>E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Paid on the CTTX path over 36 months (build + connection fee + 36 monthly bills)</t>
+        </is>
+      </c>
+      <c r="B33" s="22">
+        <f>E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Difference over the term (positive = CTTX path cheaper) - and the lodge owns the network at the end</t>
+        </is>
+      </c>
+      <c r="B34" s="28">
+        <f>E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Total 5-year saving vs Herotel (recommended path)</t>
         </is>
       </c>
-      <c r="I31" s="28">
+      <c r="I36" s="29">
         <f>G20</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>5-Year ROI (total saving as % of total upfront cash outlay)</t>
         </is>
       </c>
-      <c r="I32" s="29">
+      <c r="I37" s="30">
         <f>G21</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="C4:H4"/>
@@ -2501,14 +2557,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
@@ -2530,12 +2586,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -2549,178 +2605,212 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Annual price escalation (Herotel and Vodacom)</t>
+          <t>Annual price escalation - current provider (Herotel)</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>8% p.a.</t>
-        </is>
-      </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>Not confirmed by either party - a typical CPI-linked telecom escalation in South Africa. Editable on tab 4; change it and every formula recalculates.</t>
+          <t>8% p.a. from year 2</t>
+        </is>
+      </c>
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>Not confirmed by Herotel - a typical CPI-linked telecom escalation in South Africa. Editable on tab 4; change it and every formula recalculates. Set it to 0% and payback moves from 2 years 10 months to 3 years 4 months.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>VAT rate</t>
+          <t>Price escalation - CTTX path (Vodacom + retainer)</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C6" s="31" t="inlineStr">
-        <is>
-          <t>Current South African VAT rate.</t>
+          <t>0% for the 36-month term, then 8% p.a.</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="inlineStr">
+        <is>
+          <t>The Vodacom Business Connect 36-month contract price and the CTTX retainer are fixed for the term of the agreement. The same 8% is applied after the term ends (years 4-5) so the CTTX path is not flattered.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Managed Service Retainer</t>
+          <t>Timing of the comparison</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>R1,500/month excl. VAT</t>
-        </is>
-      </c>
-      <c r="C7" s="31" t="inlineStr">
-        <is>
-          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+          <t>Both paths start at month 1</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="inlineStr">
+        <is>
+          <t>Year 0 is the build payment only. Neither path is charged any monthly bill in year 0 - an earlier version of this model charged Herotel a full year before the build and gave the CTTX path none, which overstated the case. Corrected 28 Sept 2026.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>VAT rate</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>Current South African VAT rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Managed Service Retainer</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>R1,500/month excl. VAT</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>Contract term - Vodacom Business Connect</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>36 months</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>Confirmed 28 Sept 2026 against the CTTX Vodacom Reseller price book (Duane Forlee, Vodacom, 29 May 2026): the 36-month rate is slightly lower than 24-month. Monthly figure in this model is the confirmed 36-month client price at CTTX's standard 20% markup.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Design Assumptions</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>What's Included in the 10-Year Support</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Years 1-3: monthly remote monitoring, quarterly on-site maintenance, 24/7 emergency support, proactive performance reporting, warranty-covered equipment troubleshooting/replacement.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Years 4-10: ongoing remote monitoring, annual on-site maintenance/assessment, 24/7 support continuation, planned technology refresh, performance reporting.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>What's Excluded / Not Yet Priced</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="32" t="inlineStr">
         <is>
           <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>Any scope beyond the confirmed coverage zones (28 subscriber sites) without a signed change order.</t>
         </is>
@@ -2728,23 +2818,23 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Lead with long-term value; add payment terms and balance-sheet case
Section order is now value (04) before price (05). The R355,000 hero
number becomes one tile alongside payment terms (50% on order, 50% on
commissioning) and ownership. Adds three value cards: the build as a
capitalised asset (ex-VAT figure, recoverable input VAT, depreciable,
transfers with the property); growth on the rental model costs recurring
AP fees and a link to reach the spa vs once-off hardware on an owned
network; locked term price then no rental to renew. Workbook tab 5
records the same assumptions.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_5Year_Business_Case.xlsx
+++ b/proposals/Barefoot_5Year_Business_Case.xlsx
@@ -2563,7 +2563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2639,178 +2639,229 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Timing of the comparison</t>
+          <t>Payment terms - build</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Both paths start at month 1</t>
+          <t>50% deposit on order, 50% on commissioning</t>
         </is>
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Year 0 is the build payment only. Neither path is charged any monthly bill in year 0 - an earlier version of this model charged Herotel a full year before the build and gave the CTTX path none, which overstated the case. Corrected 28 Sept 2026.</t>
+          <t>The deposit places the equipment order and secures the allocation. Both halves fall in year 0 of the cash flow, so the model is unchanged by the split.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>VAT rate</t>
+          <t>Accounting treatment - build</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Capital expenditure (fixed asset)</t>
         </is>
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>Current South African VAT rate.</t>
+          <t>R308,696 ex VAT is capitalised as owned infrastructure on the lodge's balance sheet; the R46,304 input VAT is recoverable for a VAT-registered entity; the asset is depreciable over its working life and transfers with the property. The lodge's accountant confirms the exact treatment - this workbook does not model the tax effect (which would only improve the case).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Managed Service Retainer</t>
+          <t>Spa and future endpoints</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>R1,500/month excl. VAT</t>
+          <t>Not in the current-provider line</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+          <t>The current bill excludes the spa (not connected today). On the rental model each additional AP is ~R263/month incl. VAT (per the current invoice) plus a link to reach the spa; on the owned network it is a once-off hardware cost. Left out of the comparison deliberately - the current-provider line is therefore understated, not overstated.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>Timing of the comparison</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Both paths start at month 1</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>Year 0 is the build payment only. Neither path is charged any monthly bill in year 0 - an earlier version of this model charged Herotel a full year before the build and gave the CTTX path none, which overstated the case. Corrected 28 Sept 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>VAT rate</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Current South African VAT rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Managed Service Retainer</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>R1,500/month excl. VAT</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>Contract term - Vodacom Business Connect</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>36 months</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Confirmed 28 Sept 2026 against the CTTX Vodacom Reseller price book (Duane Forlee, Vodacom, 29 May 2026): the 36-month rate is slightly lower than 24-month. Monthly figure in this model is the confirmed 36-month client price at CTTX's standard 20% markup.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Design Assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
-        <is>
-          <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
-        <is>
-          <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
-        <is>
-          <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="32" t="inlineStr">
         <is>
-          <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
+          <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="32" t="inlineStr">
         <is>
-          <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>What's Included in the 10-Year Support</t>
+          <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="32" t="inlineStr">
         <is>
+          <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>What's Included in the 10-Year Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
           <t>Years 1-3: monthly remote monitoring, quarterly on-site maintenance, 24/7 emergency support, proactive performance reporting, warranty-covered equipment troubleshooting/replacement.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="32" t="inlineStr">
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Years 4-10: ongoing remote monitoring, annual on-site maintenance/assessment, 24/7 support continuation, planned technology refresh, performance reporting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>What's Excluded / Not Yet Priced</t>
         </is>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="32" t="inlineStr">
         <is>
-          <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="32" t="inlineStr">
-        <is>
-          <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="32" t="inlineStr">
-        <is>
-          <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
+          <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>What's Excluded / Not Yet Priced</t>
         </is>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="32" t="inlineStr">
         <is>
-          <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
+          <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>Any scope beyond the confirmed coverage zones (28 subscriber sites) without a signed change order.</t>
         </is>
@@ -2820,22 +2871,22 @@
   <mergeCells count="18">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>